<commit_message>
feat: tracker template gains header filters (follows Catchr's new sheet setup)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/catchr-job-tracker-template.xlsx
+++ b/downloads/catchr-job-tracker-template.xlsx
@@ -10,7 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jobs" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Jobs'!$A$1:$L$1000</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -13509,6 +13511,7 @@
       <c r="K1000" s="4" t="n"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:L1000"/>
   <conditionalFormatting sqref="E2:E1000">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"yes"</formula>

</xml_diff>